<commit_message>
Zmiana czesci emaili na realistyczne adresy
</commit_message>
<xml_diff>
--- a/data/xlsx/ceidg.xlsx
+++ b/data/xlsx/ceidg.xlsx
@@ -205,7 +205,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>magdalena.pawlak@astra-finance.pl</t>
+          <t>magdalena.pawlak@interia.pl</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -297,7 +297,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>r.michalski@biuro.pl</t>
+          <t>r.michalski@o2.pl</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -389,7 +389,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>krol.agnieszka@poczta.pl</t>
+          <t>krol.agnieszka@brak-domeny</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -481,7 +481,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>wojciechwieczorek@mail.pl</t>
+          <t>wojciechwieczorek@outlook.com</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>justyna_jablonska@nova-data.pl</t>
+          <t>justyna_jablonska@yahoo.com</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>piotr.witkowski95@wp.pl</t>
+          <t>piotr.witkowski95@icloud.com</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>m.stepien@proton.me</t>
+          <t>m.stepien@localhost</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>baran.joanna@silesia-invest.pl</t>
+          <t>baran.joanna@onet.pl</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>pawelrutkowski@poczta.pl</t>
+          <t>pawelrutkowski@interia.pl</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>magdalena_gorska@mail.pl</t>
+          <t>magdalena_gorska@o2.pl</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>robert.sikora72@onet.pl</t>
+          <t>robert.sikora72@proton.me</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>agnieszka.ostrowska@helios-markets.pl</t>
+          <t>agnieszka.ostrowska@brak-domeny</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>w.tomaszewski@gmail.com</t>
+          <t>w.tomaszewski@yahoo.com</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>zajac.justyna@proton.me</t>
+          <t>zajac.justyna@icloud.com</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>piotrpietrzak@biuro.pl</t>
+          <t>piotrpietrzak@gmail.com</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>maria_wojcicka@polaris-capital.pl</t>
+          <t>maria_wojcicka@wp.pl</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>michal.czarnecki78@mail.pl</t>
+          <t>michal.czarnecki78@localhost</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>joanna.lis@onet.pl</t>
+          <t>joanna.lis@interia.pl</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>p.kolodziej@wp.pl</t>
+          <t>p.kolodziej@o2.pl</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>kaczmarek.magdalena@astra-finance.pl</t>
+          <t>kaczmarek.magdalena@proton.me</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>robertpiatek@proton.me</t>
+          <t>robertpiatek@outlook.com</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>agnieszka_sadowska@biuro.pl</t>
+          <t>agnieszka_sadowska@brak-domeny</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>wojciech.wlodarczyk84@poczta.pl</t>
+          <t>wojciech.wlodarczyk84@icloud.com</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>justyna.borkowska@nova-data.pl</t>
+          <t>justyna.borkowska@gmail.com</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>p.kowalski@onet.pl</t>
+          <t>p.kowalski@wp.pl</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>nowacka.maria@wp.pl</t>
+          <t>nowacka.maria@onet.pl</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>joanna_wojcik@silesia-invest.pl</t>
+          <t>joanna_wojcik@localhost</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>pawel.kowalczyk90@biuro.pl</t>
+          <t>pawel.kowalczyk90@o2.pl</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>magdalena.kaminska@poczta.pl</t>
+          <t>magdalena.kaminska@proton.me</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>r.lewandowski@mail.pl</t>
+          <t>r.lewandowski@outlook.com</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3149,7 +3149,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>zielinska.agnieszka@helios-markets.pl</t>
+          <t>zielinska.agnieszka@yahoo.com</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>wojciechszymanski@wp.pl</t>
+          <t>wojciechszymanski@brak-domeny</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>piotr.mazur96@proton.me</t>
+          <t>piotr.mazur96@wp.pl</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>maria.krawczyk@polaris-capital.pl</t>
+          <t>maria.krawczyk@onet.pl</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>m.wozniak@poczta.pl</t>
+          <t>m.wozniak@interia.pl</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>jankowska.joanna@mail.pl</t>
+          <t>jankowska.joanna@localhost</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>pawelgrabowski@onet.pl</t>
+          <t>pawelgrabowski@proton.me</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>magdalena_pawlak@astra-finance.pl</t>
+          <t>magdalena_pawlak@outlook.com</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -3977,7 +3977,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>robert.michalski73@gmail.com</t>
+          <t>robert.michalski73@yahoo.com</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>agnieszka.krol@proton.me</t>
+          <t>agnieszka.krol@icloud.com</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>w.wieczorek@biuro.pl</t>
+          <t>w.wieczorek@brak-domeny</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>jablonska.justyna@nova-data.pl</t>
+          <t>jablonska.justyna@wp.pl</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4345,7 +4345,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>piotrwitkowski@mail.pl</t>
+          <t>piotrwitkowski@onet.pl</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4437,7 +4437,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>maria_walczak@onet.pl</t>
+          <t>maria_walczak@interia.pl</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -4529,7 +4529,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>michal.stepien79@wp.pl</t>
+          <t>michal.stepien79@o2.pl</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4621,7 +4621,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>joanna.baran@silesia-invest.pl</t>
+          <t>joanna.baran@localhost</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>p.rutkowski@proton.me</t>
+          <t>p.rutkowski@outlook.com</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>gorska.magdalena@biuro.pl</t>
+          <t>gorska.magdalena@yahoo.com</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>robertsikora@poczta.pl</t>
+          <t>robertsikora@icloud.com</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>agnieszka_ostrowska@helios-markets.pl</t>
+          <t>agnieszka_ostrowska@gmail.com</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>wojciech.tomaszewski85@onet.pl</t>
+          <t>wojciech.tomaszewski85@wp.pl</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5173,7 +5173,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>justyna.zajac@wp.pl</t>
+          <t>justyna.zajac@domena..pl</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>p.pietrzak@gmail.com</t>
+          <t>p.pietrzak@interia.pl</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5357,7 +5357,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>wojcicka.maria@polaris-capital.pl</t>
+          <t>wojcicka.maria@o2.pl</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5449,7 +5449,7 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>michalczarnecki@biuro.pl</t>
+          <t>michalczarnecki@proton.me</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -5541,7 +5541,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>joanna_lis@poczta.pl</t>
+          <t>joanna_lis@outlook.com</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>pawel.kolodziej91@mail.pl</t>
+          <t>pawel.kolodziej91@.pl</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5725,7 +5725,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>magdalena.kaczmarek@astra-finance.pl</t>
+          <t>magdalena.kaczmarek@icloud.com</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -5817,7 +5817,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>r.piatek@wp.pl</t>
+          <t>r.piatek@gmail.com</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -5909,7 +5909,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>sadowska.agnieszka@gmail.com</t>
+          <t>sadowska.agnieszka@wp.pl</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -6001,7 +6001,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>wojciechwlodarczyk@proton.me</t>
+          <t>wojciechwlodarczyk@onet.pl</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -6093,7 +6093,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>justyna_borkowska@nova-data.pl</t>
+          <t>justyna_borkowska@domena..pl</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6185,7 +6185,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>piotr.kowalski97@poczta.pl</t>
+          <t>piotr.kowalski97@o2.pl</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6277,7 +6277,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>maria.nowacka@mail.pl</t>
+          <t>maria.nowacka@proton.me</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -6369,7 +6369,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>m.wisniewski@onet.pl</t>
+          <t>m.wisniewski@outlook.com</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -6461,7 +6461,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>wojcik.joanna@silesia-invest.pl</t>
+          <t>wojcik.joanna@yahoo.com</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>pawelkowalczyk@gmail.com</t>
+          <t>pawelkowalczyk@.pl</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -6645,7 +6645,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>magdalena_kaminska@proton.me</t>
+          <t>magdalena_kaminska@gmail.com</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -6737,7 +6737,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>robert.lewandowski74@biuro.pl</t>
+          <t>robert.lewandowski74@wp.pl</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -6829,7 +6829,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>agnieszka.zielinska@helios-markets.pl</t>
+          <t>agnieszka.zielinska@onet.pl</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>w.szymanski@mail.pl</t>
+          <t>w.szymanski@interia.pl</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -7013,7 +7013,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>dabrowska.justyna@onet.pl</t>
+          <t>dabrowska.justyna@domena..pl</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -7105,7 +7105,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>piotrmazur@wp.pl</t>
+          <t>piotrmazur@proton.me</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -7197,7 +7197,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>maria_krawczyk@polaris-capital.pl</t>
+          <t>maria_krawczyk@outlook.com</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -7289,7 +7289,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>michal.wozniak80@proton.me</t>
+          <t>michal.wozniak80@yahoo.com</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -7381,7 +7381,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>joanna.jankowska@biuro.pl</t>
+          <t>joanna.jankowska@icloud.com</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -7473,7 +7473,7 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>p.grabowski@poczta.pl</t>
+          <t>p.grabowski@.pl</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -7565,7 +7565,7 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>pawlak.magdalena@astra-finance.pl</t>
+          <t>pawlak.magdalena@wp.pl</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -7841,7 +7841,7 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>wojciech.wieczorek86@gmail.com</t>
+          <t>wojciech.wieczorek86@interia.pl</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
@@ -7933,7 +7933,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>justyna.jablonska@nova-data.pl</t>
+          <t>justyna.jablonska@o2.pl</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
@@ -8025,7 +8025,7 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>p.witkowski@biuro.pl</t>
+          <t>p.witkowski@domena..pl</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -8117,7 +8117,7 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>walczak.maria@poczta.pl</t>
+          <t>walczak.maria@outlook.com</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -8209,7 +8209,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>michalstepien@mail.pl</t>
+          <t>michalstepien@yahoo.com</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>joanna_baran@silesia-invest.pl</t>
+          <t>joanna_baran@icloud.com</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -8393,7 +8393,7 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>pawel.rutkowski92@wp.pl</t>
+          <t>pawel.rutkowski92@gmail.com</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
@@ -8485,7 +8485,7 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>magdalena.gorska@gmail.com</t>
+          <t>magdalena.gorska@.pl</t>
         </is>
       </c>
       <c r="R92" t="inlineStr">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>r.sikora@proton.me</t>
+          <t>r.sikora@onet.pl</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
@@ -8669,7 +8669,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>ostrowska.agnieszka@helios-markets.pl</t>
+          <t>ostrowska.agnieszka@interia.pl</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>wojciechtomaszewski@poczta.pl</t>
+          <t>wojciechtomaszewski@o2.pl</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
@@ -8853,7 +8853,7 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>justyna_zajac@mail.pl</t>
+          <t>justyna_zajac@proton.me</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">
@@ -8945,7 +8945,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>piotr.pietrzak98@onet.pl</t>
+          <t>piotr.pietrzak98@domena..pl</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -9037,7 +9037,7 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>maria.wojcicka@polaris-capital.pl</t>
+          <t>maria.wojcicka@yahoo.com</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>m.czarnecki@gmail.com</t>
+          <t>m.czarnecki@icloud.com</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
@@ -9221,7 +9221,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>lis.joanna@proton.me</t>
+          <t>lis.joanna@gmail.com</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -9313,7 +9313,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>pawelkolodziej@biuro.pl</t>
+          <t>pawelkolodziej@wp.pl</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -9405,7 +9405,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>magdalena_kaczmarek@astra-finance.pl</t>
+          <t>magdalena_kaczmarek@.pl</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -9497,7 +9497,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>robert.piatek75@mail.pl</t>
+          <t>robert.piatek75@interia.pl</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -9589,7 +9589,7 @@
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>agnieszka.sadowska@onet.pl</t>
+          <t>agnieszka.sadowska@o2.pl</t>
         </is>
       </c>
       <c r="R104" t="inlineStr">
@@ -9681,7 +9681,7 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>w.wlodarczyk@wp.pl</t>
+          <t>w.wlodarczyk@proton.me</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
@@ -9773,7 +9773,7 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>borkowska.justyna@nova-data.pl</t>
+          <t>borkowska.justyna@outlook.com</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
@@ -9865,7 +9865,7 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>piotrkowalski@proton.me</t>
+          <t>piotrkowalski@domena..pl</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -9957,7 +9957,7 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>maria_nowacka@biuro.pl</t>
+          <t>maria_nowacka@icloud.com</t>
         </is>
       </c>
       <c r="R108" t="inlineStr">
@@ -10049,7 +10049,7 @@
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>michal.wisniewski81@poczta.pl</t>
+          <t>michal.wisniewski81@gmail.com</t>
         </is>
       </c>
       <c r="R109" t="inlineStr">
@@ -10141,7 +10141,7 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>joanna.wojcik@silesia-invest.pl</t>
+          <t>joanna.wojcik@wp.pl</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
@@ -10325,7 +10325,7 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>kaminska.magdalena@wp.pl</t>
+          <t>kaminska.magdalena@.pl</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -10417,7 +10417,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>robertlewandowski@gmail.com</t>
+          <t>robertlewandowski@o2.pl</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>agnieszka_zielinska@helios-markets.pl</t>
+          <t>agnieszka_zielinska@proton.me</t>
         </is>
       </c>
       <c r="R114" t="inlineStr">
@@ -10601,7 +10601,7 @@
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>wojciech.szymanski87@biuro.pl</t>
+          <t>wojciech.szymanski87@outlook.com</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -10693,7 +10693,7 @@
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>justyna.dabrowska@poczta.pl</t>
+          <t>justyna.dabrowska@yahoo.com</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -10785,7 +10785,7 @@
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>p.mazur@mail.pl</t>
+          <t>p.mazur@domena..pl</t>
         </is>
       </c>
       <c r="R117" t="inlineStr">
@@ -10877,7 +10877,7 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>krawczyk.maria@polaris-capital.pl</t>
+          <t>krawczyk.maria@gmail.com</t>
         </is>
       </c>
       <c r="R118" t="inlineStr">
@@ -11061,7 +11061,7 @@
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>joanna_jankowska@gmail.com</t>
+          <t>joanna_jankowska@onet.pl</t>
         </is>
       </c>
       <c r="R120" t="inlineStr">
@@ -11153,7 +11153,7 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>pawel.grabowski93@proton.me</t>
+          <t>pawel.grabowski93@interia.pl</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
@@ -11245,7 +11245,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>magdalena.pawlak@astra-finance.pl</t>
+          <t>magdalena.pawlak@.pl</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
@@ -11337,7 +11337,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>r.michalski@poczta.pl</t>
+          <t>r.michalski@proton.me</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
@@ -11429,7 +11429,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>krol.agnieszka@mail.pl</t>
+          <t>krol.agnieszka@outlook.com</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
@@ -11521,7 +11521,7 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>wojciechwieczorek@onet.pl</t>
+          <t>wojciechwieczorek@yahoo.com</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
@@ -11613,7 +11613,7 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>justyna_jablonska@nova-data.pl</t>
+          <t>justyna_jablonska@icloud.com</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
@@ -11705,7 +11705,7 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>piotr.witkowski70@gmail.com</t>
+          <t>piotr.witkowski70@domena..pl</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
@@ -11797,7 +11797,7 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>maria.walczak@proton.me</t>
+          <t>maria.walczak@wp.pl</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
@@ -11981,7 +11981,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>baran.joanna@silesia-invest.pl</t>
+          <t>baran.joanna@onet.pl</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
@@ -12073,7 +12073,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>pawelrutkowski@mail.pl</t>
+          <t>pawelrutkowski@interia.pl</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
@@ -12165,7 +12165,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>magdalena_gorska@onet.pl</t>
+          <t>magdalena_gorska@o2.pl</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -12257,7 +12257,7 @@
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>robert.sikora76@wp.pl</t>
+          <t>robert.sikora76@.pl</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
@@ -12349,7 +12349,7 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>agnieszka.ostrowska@helios-markets.pl</t>
+          <t>agnieszka.ostrowska@outlook.com</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
@@ -12441,7 +12441,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>w.tomaszewski@proton.me</t>
+          <t>w.tomaszewski@yahoo.com</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -12533,7 +12533,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>zajac.justyna@biuro.pl</t>
+          <t>zajac.justyna@icloud.com</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
@@ -12625,7 +12625,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>piotrpietrzak@poczta.pl</t>
+          <t>piotrpietrzak@gmail.com</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -12717,7 +12717,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>maria_wojcicka@polaris-capital.pl</t>
+          <t>maria_wojcicka@domena..pl</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
@@ -12901,7 +12901,7 @@
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>joanna.lis@wp.pl</t>
+          <t>joanna.lis@interia.pl</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
@@ -12993,7 +12993,7 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>p.kolodziej@gmail.com</t>
+          <t>p.kolodziej@o2.pl</t>
         </is>
       </c>
       <c r="R141" t="inlineStr">
@@ -13085,7 +13085,7 @@
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>kaczmarek.magdalena@astra-finance.pl</t>
+          <t>kaczmarek.magdalena@proton.me</t>
         </is>
       </c>
       <c r="R142" t="inlineStr">
@@ -13177,7 +13177,7 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>robertpiatek@biuro.pl</t>
+          <t>robertpiatek@.pl</t>
         </is>
       </c>
       <c r="R143" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>agnieszka_sadowska@poczta.pl</t>
+          <t>agnieszka_sadowska@yahoo.com</t>
         </is>
       </c>
       <c r="R144" t="inlineStr">
@@ -13361,7 +13361,7 @@
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>wojciech.wlodarczyk88@mail.pl</t>
+          <t>wojciech.wlodarczyk88@icloud.com</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
@@ -13453,7 +13453,7 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>justyna.borkowska@nova-data.pl</t>
+          <t>justyna.borkowska@gmail.com</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
@@ -13637,7 +13637,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>nowacka.maria@gmail.com</t>
+          <t>nowacka.maria@domena..pl</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
@@ -13729,7 +13729,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>michalwisniewski@proton.me</t>
+          <t>michalwisniewski@interia.pl</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
@@ -13821,7 +13821,7 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>joanna_wojcik@silesia-invest.pl</t>
+          <t>joanna_wojcik@o2.pl</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
@@ -13913,7 +13913,7 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>pawel.kowalczyk94@poczta.pl</t>
+          <t>pawel.kowalczyk94@proton.me</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
@@ -14005,7 +14005,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>magdalena.kaminska@mail.pl</t>
+          <t>magdalena.kaminska@outlook.com</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
@@ -14097,7 +14097,7 @@
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>r.lewandowski@onet.pl</t>
+          <t>r.lewandowski@yahoo.com</t>
         </is>
       </c>
       <c r="R153" t="inlineStr">
@@ -14189,7 +14189,7 @@
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>zielinska.agnieszka@helios-markets.pl</t>
+          <t>zielinska.agnieszka@wp</t>
         </is>
       </c>
       <c r="R154" t="inlineStr">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>justyna_dabrowska@proton.me</t>
+          <t>justyna_dabrowska@wp.pl</t>
         </is>
       </c>
       <c r="R156" t="inlineStr">
@@ -14465,7 +14465,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>piotr.mazur71@biuro.pl</t>
+          <t>piotr.mazur71@onet.pl</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
@@ -14557,7 +14557,7 @@
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>maria.krawczyk@polaris-capital.pl</t>
+          <t>maria.krawczyk@interia.pl</t>
         </is>
       </c>
       <c r="R158" t="inlineStr">
@@ -14649,7 +14649,7 @@
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>m.wozniak@mail.pl</t>
+          <t>@m.wozniak.invalid</t>
         </is>
       </c>
       <c r="R159" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>jankowska.joanna@onet.pl</t>
+          <t>jankowska.joanna@proton.me</t>
         </is>
       </c>
       <c r="R160" t="inlineStr">
@@ -14833,7 +14833,7 @@
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>pawelgrabowski@wp.pl</t>
+          <t>pawelgrabowski@outlook.com</t>
         </is>
       </c>
       <c r="R161" t="inlineStr">
@@ -14925,7 +14925,7 @@
       </c>
       <c r="Q162" t="inlineStr">
         <is>
-          <t>magdalena_pawlak@astra-finance.pl</t>
+          <t>magdalena_pawlak@yahoo.com</t>
         </is>
       </c>
       <c r="R162" t="inlineStr">
@@ -15017,7 +15017,7 @@
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>robert.michalski77@proton.me</t>
+          <t>robert.michalski77@icloud.com</t>
         </is>
       </c>
       <c r="R163" t="inlineStr">
@@ -15109,7 +15109,7 @@
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>agnieszka.krol@biuro.pl</t>
+          <t>agnieszka.krol@wp</t>
         </is>
       </c>
       <c r="R164" t="inlineStr">
@@ -15201,7 +15201,7 @@
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>w.wieczorek@poczta.pl</t>
+          <t>w.wieczorek@wp.pl</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
@@ -15293,7 +15293,7 @@
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>jablonska.justyna@nova-data.pl</t>
+          <t>jablonska.justyna@onet.pl</t>
         </is>
       </c>
       <c r="R166" t="inlineStr">
@@ -15385,7 +15385,7 @@
       </c>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>piotrwitkowski@onet.pl</t>
+          <t>piotrwitkowski@interia.pl</t>
         </is>
       </c>
       <c r="R167" t="inlineStr">
@@ -15477,7 +15477,7 @@
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>maria_walczak@wp.pl</t>
+          <t>maria_walczak@o2.pl</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
@@ -15569,7 +15569,7 @@
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>michal.stepien83@gmail.com</t>
+          <t>@michal.stepien83.invalid</t>
         </is>
       </c>
       <c r="R169" t="inlineStr">
@@ -15661,7 +15661,7 @@
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>joanna.baran@silesia-invest.pl</t>
+          <t>joanna.baran@outlook.com</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
@@ -15753,7 +15753,7 @@
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>p.rutkowski@biuro.pl</t>
+          <t>p.rutkowski@yahoo.com</t>
         </is>
       </c>
       <c r="R171" t="inlineStr">
@@ -15845,7 +15845,7 @@
       </c>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>gorska.magdalena@poczta.pl</t>
+          <t>gorska.magdalena@icloud.com</t>
         </is>
       </c>
       <c r="R172" t="inlineStr">
@@ -15937,7 +15937,7 @@
       </c>
       <c r="Q173" t="inlineStr">
         <is>
-          <t>robertsikora@mail.pl</t>
+          <t>robertsikora@gmail.com</t>
         </is>
       </c>
       <c r="R173" t="inlineStr">
@@ -16029,7 +16029,7 @@
       </c>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>agnieszka_ostrowska@helios-markets.pl</t>
+          <t>agnieszka_ostrowska@wp</t>
         </is>
       </c>
       <c r="R174" t="inlineStr">
@@ -16121,7 +16121,7 @@
       </c>
       <c r="Q175" t="inlineStr">
         <is>
-          <t>wojciech.tomaszewski89@wp.pl</t>
+          <t>wojciech.tomaszewski89@onet.pl</t>
         </is>
       </c>
       <c r="R175" t="inlineStr">
@@ -16213,7 +16213,7 @@
       </c>
       <c r="Q176" t="inlineStr">
         <is>
-          <t>justyna.zajac@gmail.com</t>
+          <t>justyna.zajac@interia.pl</t>
         </is>
       </c>
       <c r="R176" t="inlineStr">
@@ -16305,7 +16305,7 @@
       </c>
       <c r="Q177" t="inlineStr">
         <is>
-          <t>p.pietrzak@proton.me</t>
+          <t>p.pietrzak@o2.pl</t>
         </is>
       </c>
       <c r="R177" t="inlineStr">
@@ -16397,7 +16397,7 @@
       </c>
       <c r="Q178" t="inlineStr">
         <is>
-          <t>wojcicka.maria@polaris-capital.pl</t>
+          <t>wojcicka.maria@proton.me</t>
         </is>
       </c>
       <c r="R178" t="inlineStr">
@@ -16489,7 +16489,7 @@
       </c>
       <c r="Q179" t="inlineStr">
         <is>
-          <t>michalczarnecki@poczta.pl</t>
+          <t>@michalczarnecki.invalid</t>
         </is>
       </c>
       <c r="R179" t="inlineStr">
@@ -16581,7 +16581,7 @@
       </c>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>joanna_lis@mail.pl</t>
+          <t>joanna_lis@yahoo.com</t>
         </is>
       </c>
       <c r="R180" t="inlineStr">
@@ -16673,7 +16673,7 @@
       </c>
       <c r="Q181" t="inlineStr">
         <is>
-          <t>pawel.kolodziej95@onet.pl</t>
+          <t>pawel.kolodziej95@icloud.com</t>
         </is>
       </c>
       <c r="R181" t="inlineStr">
@@ -16765,7 +16765,7 @@
       </c>
       <c r="Q182" t="inlineStr">
         <is>
-          <t>magdalena.kaczmarek@astra-finance.pl</t>
+          <t>magdalena.kaczmarek@gmail.com</t>
         </is>
       </c>
       <c r="R182" t="inlineStr">
@@ -16857,7 +16857,7 @@
       </c>
       <c r="Q183" t="inlineStr">
         <is>
-          <t>r.piatek@gmail.com</t>
+          <t>r.piatek@wp.pl</t>
         </is>
       </c>
       <c r="R183" t="inlineStr">
@@ -16949,7 +16949,7 @@
       </c>
       <c r="Q184" t="inlineStr">
         <is>
-          <t>sadowska.agnieszka@proton.me</t>
+          <t>sadowska.agnieszka@wp</t>
         </is>
       </c>
       <c r="R184" t="inlineStr">
@@ -17041,7 +17041,7 @@
       </c>
       <c r="Q185" t="inlineStr">
         <is>
-          <t>wojciechwlodarczyk@biuro.pl</t>
+          <t>wojciechwlodarczyk@interia.pl</t>
         </is>
       </c>
       <c r="R185" t="inlineStr">
@@ -17133,7 +17133,7 @@
       </c>
       <c r="Q186" t="inlineStr">
         <is>
-          <t>justyna_borkowska@nova-data.pl</t>
+          <t>justyna_borkowska@o2.pl</t>
         </is>
       </c>
       <c r="R186" t="inlineStr">
@@ -17225,7 +17225,7 @@
       </c>
       <c r="Q187" t="inlineStr">
         <is>
-          <t>piotr.kowalski72@mail.pl</t>
+          <t>piotr.kowalski72@proton.me</t>
         </is>
       </c>
       <c r="R187" t="inlineStr">
@@ -17317,7 +17317,7 @@
       </c>
       <c r="Q188" t="inlineStr">
         <is>
-          <t>maria.nowacka@onet.pl</t>
+          <t>maria.nowacka@outlook.com</t>
         </is>
       </c>
       <c r="R188" t="inlineStr">
@@ -17409,7 +17409,7 @@
       </c>
       <c r="Q189" t="inlineStr">
         <is>
-          <t>m.wisniewski@wp.pl</t>
+          <t>@m.wisniewski.invalid</t>
         </is>
       </c>
       <c r="R189" t="inlineStr">
@@ -17501,7 +17501,7 @@
       </c>
       <c r="Q190" t="inlineStr">
         <is>
-          <t>wojcik.joanna@silesia-invest.pl</t>
+          <t>wojcik.joanna@icloud.com</t>
         </is>
       </c>
       <c r="R190" t="inlineStr">
@@ -17593,7 +17593,7 @@
       </c>
       <c r="Q191" t="inlineStr">
         <is>
-          <t>pawelkowalczyk@proton.me</t>
+          <t>pawelkowalczyk@gmail.com</t>
         </is>
       </c>
       <c r="R191" t="inlineStr">
@@ -17685,7 +17685,7 @@
       </c>
       <c r="Q192" t="inlineStr">
         <is>
-          <t>magdalena_kaminska@biuro.pl</t>
+          <t>magdalena_kaminska@wp.pl</t>
         </is>
       </c>
       <c r="R192" t="inlineStr">
@@ -17777,7 +17777,7 @@
       </c>
       <c r="Q193" t="inlineStr">
         <is>
-          <t>robert.lewandowski78@poczta.pl</t>
+          <t>robert.lewandowski78@onet.pl</t>
         </is>
       </c>
       <c r="R193" t="inlineStr">
@@ -17869,7 +17869,7 @@
       </c>
       <c r="Q194" t="inlineStr">
         <is>
-          <t>agnieszka.zielinska@helios-markets.pl</t>
+          <t>agnieszka.zielinska@wp</t>
         </is>
       </c>
       <c r="R194" t="inlineStr">
@@ -17961,7 +17961,7 @@
       </c>
       <c r="Q195" t="inlineStr">
         <is>
-          <t>w.szymanski@onet.pl</t>
+          <t>w.szymanski@o2.pl</t>
         </is>
       </c>
       <c r="R195" t="inlineStr">
@@ -18053,7 +18053,7 @@
       </c>
       <c r="Q196" t="inlineStr">
         <is>
-          <t>dabrowska.justyna@wp.pl</t>
+          <t>dabrowska.justyna@proton.me</t>
         </is>
       </c>
       <c r="R196" t="inlineStr">
@@ -18145,7 +18145,7 @@
       </c>
       <c r="Q197" t="inlineStr">
         <is>
-          <t>piotrmazur@gmail.com</t>
+          <t>piotrmazur@outlook.com</t>
         </is>
       </c>
       <c r="R197" t="inlineStr">
@@ -18237,7 +18237,7 @@
       </c>
       <c r="Q198" t="inlineStr">
         <is>
-          <t>maria_krawczyk@polaris-capital.pl</t>
+          <t>maria_krawczyk@yahoo.com</t>
         </is>
       </c>
       <c r="R198" t="inlineStr">
@@ -18329,7 +18329,7 @@
       </c>
       <c r="Q199" t="inlineStr">
         <is>
-          <t>michal.wozniak84@biuro.pl</t>
+          <t>@michal.wozniak84.invalid</t>
         </is>
       </c>
       <c r="R199" t="inlineStr">
@@ -18421,7 +18421,7 @@
       </c>
       <c r="Q200" t="inlineStr">
         <is>
-          <t>joanna.jankowska@poczta.pl</t>
+          <t>joanna.jankowska@gmail.com</t>
         </is>
       </c>
       <c r="R200" t="inlineStr">
@@ -18513,7 +18513,7 @@
       </c>
       <c r="Q201" t="inlineStr">
         <is>
-          <t>p.grabowski@mail.pl</t>
+          <t>p.grabowski@wp.pl</t>
         </is>
       </c>
       <c r="R201" t="inlineStr">

</xml_diff>

<commit_message>
Email address fixes (#22)
* Zmiana czesci emaili na realistyczne adresy

* Poprawa walidacji istnienia domen email
</commit_message>
<xml_diff>
--- a/data/xlsx/ceidg.xlsx
+++ b/data/xlsx/ceidg.xlsx
@@ -205,7 +205,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>magdalena.pawlak@astra-finance.pl</t>
+          <t>magdalena.pawlak@interia.pl</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -297,7 +297,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>r.michalski@biuro.pl</t>
+          <t>r.michalski@o2.pl</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -389,7 +389,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>krol.agnieszka@poczta.pl</t>
+          <t>krol.agnieszka@brak-domeny</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -481,7 +481,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>wojciechwieczorek@mail.pl</t>
+          <t>wojciechwieczorek@outlook.com</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>justyna_jablonska@nova-data.pl</t>
+          <t>justyna_jablonska@yahoo.com</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>piotr.witkowski95@wp.pl</t>
+          <t>piotr.witkowski95@icloud.com</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>m.stepien@proton.me</t>
+          <t>m.stepien@localhost</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>baran.joanna@silesia-invest.pl</t>
+          <t>baran.joanna@onet.pl</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>pawelrutkowski@poczta.pl</t>
+          <t>pawelrutkowski@interia.pl</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>magdalena_gorska@mail.pl</t>
+          <t>magdalena_gorska@o2.pl</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>robert.sikora72@onet.pl</t>
+          <t>robert.sikora72@proton.me</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>agnieszka.ostrowska@helios-markets.pl</t>
+          <t>agnieszka.ostrowska@brak-domeny</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>w.tomaszewski@gmail.com</t>
+          <t>w.tomaszewski@yahoo.com</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>zajac.justyna@proton.me</t>
+          <t>zajac.justyna@icloud.com</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>piotrpietrzak@biuro.pl</t>
+          <t>piotrpietrzak@gmail.com</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>maria_wojcicka@polaris-capital.pl</t>
+          <t>maria_wojcicka@wp.pl</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>michal.czarnecki78@mail.pl</t>
+          <t>michal.czarnecki78@localhost</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>joanna.lis@onet.pl</t>
+          <t>joanna.lis@interia.pl</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>p.kolodziej@wp.pl</t>
+          <t>p.kolodziej@o2.pl</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>kaczmarek.magdalena@astra-finance.pl</t>
+          <t>kaczmarek.magdalena@proton.me</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>robertpiatek@proton.me</t>
+          <t>robertpiatek@outlook.com</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>agnieszka_sadowska@biuro.pl</t>
+          <t>agnieszka_sadowska@brak-domeny</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>wojciech.wlodarczyk84@poczta.pl</t>
+          <t>wojciech.wlodarczyk84@icloud.com</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>justyna.borkowska@nova-data.pl</t>
+          <t>justyna.borkowska@gmail.com</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>p.kowalski@onet.pl</t>
+          <t>p.kowalski@wp.pl</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>nowacka.maria@wp.pl</t>
+          <t>nowacka.maria@onet.pl</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>joanna_wojcik@silesia-invest.pl</t>
+          <t>joanna_wojcik@localhost</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>pawel.kowalczyk90@biuro.pl</t>
+          <t>pawel.kowalczyk90@o2.pl</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>magdalena.kaminska@poczta.pl</t>
+          <t>magdalena.kaminska@proton.me</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>r.lewandowski@mail.pl</t>
+          <t>r.lewandowski@outlook.com</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3149,7 +3149,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>zielinska.agnieszka@helios-markets.pl</t>
+          <t>zielinska.agnieszka@yahoo.com</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>wojciechszymanski@wp.pl</t>
+          <t>wojciechszymanski@brak-domeny</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>piotr.mazur96@proton.me</t>
+          <t>piotr.mazur96@wp.pl</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>maria.krawczyk@polaris-capital.pl</t>
+          <t>maria.krawczyk@onet.pl</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>m.wozniak@poczta.pl</t>
+          <t>m.wozniak@interia.pl</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>jankowska.joanna@mail.pl</t>
+          <t>jankowska.joanna@localhost</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>pawelgrabowski@onet.pl</t>
+          <t>pawelgrabowski@proton.me</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>magdalena_pawlak@astra-finance.pl</t>
+          <t>magdalena_pawlak@outlook.com</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -3977,7 +3977,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>robert.michalski73@gmail.com</t>
+          <t>robert.michalski73@yahoo.com</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>agnieszka.krol@proton.me</t>
+          <t>agnieszka.krol@icloud.com</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>w.wieczorek@biuro.pl</t>
+          <t>w.wieczorek@brak-domeny</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>jablonska.justyna@nova-data.pl</t>
+          <t>jablonska.justyna@wp.pl</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4345,7 +4345,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>piotrwitkowski@mail.pl</t>
+          <t>piotrwitkowski@onet.pl</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4437,7 +4437,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>maria_walczak@onet.pl</t>
+          <t>maria_walczak@interia.pl</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -4529,7 +4529,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>michal.stepien79@wp.pl</t>
+          <t>michal.stepien79@o2.pl</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4621,7 +4621,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>joanna.baran@silesia-invest.pl</t>
+          <t>joanna.baran@localhost</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>p.rutkowski@proton.me</t>
+          <t>p.rutkowski@outlook.com</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>gorska.magdalena@biuro.pl</t>
+          <t>gorska.magdalena@yahoo.com</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>robertsikora@poczta.pl</t>
+          <t>robertsikora@icloud.com</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>agnieszka_ostrowska@helios-markets.pl</t>
+          <t>agnieszka_ostrowska@gmail.com</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>wojciech.tomaszewski85@onet.pl</t>
+          <t>wojciech.tomaszewski85@wp.pl</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5173,7 +5173,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>justyna.zajac@wp.pl</t>
+          <t>justyna.zajac@domena..pl</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>p.pietrzak@gmail.com</t>
+          <t>p.pietrzak@interia.pl</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5357,7 +5357,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>wojcicka.maria@polaris-capital.pl</t>
+          <t>wojcicka.maria@o2.pl</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5449,7 +5449,7 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>michalczarnecki@biuro.pl</t>
+          <t>michalczarnecki@proton.me</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -5541,7 +5541,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>joanna_lis@poczta.pl</t>
+          <t>joanna_lis@outlook.com</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>pawel.kolodziej91@mail.pl</t>
+          <t>pawel.kolodziej91@.pl</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5725,7 +5725,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>magdalena.kaczmarek@astra-finance.pl</t>
+          <t>magdalena.kaczmarek@icloud.com</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -5817,7 +5817,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>r.piatek@wp.pl</t>
+          <t>r.piatek@gmail.com</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -5909,7 +5909,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>sadowska.agnieszka@gmail.com</t>
+          <t>sadowska.agnieszka@wp.pl</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -6001,7 +6001,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>wojciechwlodarczyk@proton.me</t>
+          <t>wojciechwlodarczyk@onet.pl</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -6093,7 +6093,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>justyna_borkowska@nova-data.pl</t>
+          <t>justyna_borkowska@domena..pl</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6185,7 +6185,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>piotr.kowalski97@poczta.pl</t>
+          <t>piotr.kowalski97@o2.pl</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6277,7 +6277,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>maria.nowacka@mail.pl</t>
+          <t>maria.nowacka@proton.me</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -6369,7 +6369,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>m.wisniewski@onet.pl</t>
+          <t>m.wisniewski@outlook.com</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -6461,7 +6461,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>wojcik.joanna@silesia-invest.pl</t>
+          <t>wojcik.joanna@yahoo.com</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>pawelkowalczyk@gmail.com</t>
+          <t>pawelkowalczyk@.pl</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -6645,7 +6645,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>magdalena_kaminska@proton.me</t>
+          <t>magdalena_kaminska@gmail.com</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -6737,7 +6737,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>robert.lewandowski74@biuro.pl</t>
+          <t>robert.lewandowski74@wp.pl</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -6829,7 +6829,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>agnieszka.zielinska@helios-markets.pl</t>
+          <t>agnieszka.zielinska@onet.pl</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>w.szymanski@mail.pl</t>
+          <t>w.szymanski@interia.pl</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -7013,7 +7013,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>dabrowska.justyna@onet.pl</t>
+          <t>dabrowska.justyna@domena..pl</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -7105,7 +7105,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>piotrmazur@wp.pl</t>
+          <t>piotrmazur@proton.me</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -7197,7 +7197,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>maria_krawczyk@polaris-capital.pl</t>
+          <t>maria_krawczyk@outlook.com</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -7289,7 +7289,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>michal.wozniak80@proton.me</t>
+          <t>michal.wozniak80@yahoo.com</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -7381,7 +7381,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>joanna.jankowska@biuro.pl</t>
+          <t>joanna.jankowska@icloud.com</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -7473,7 +7473,7 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>p.grabowski@poczta.pl</t>
+          <t>p.grabowski@.pl</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -7565,7 +7565,7 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>pawlak.magdalena@astra-finance.pl</t>
+          <t>pawlak.magdalena@wp.pl</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -7841,7 +7841,7 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>wojciech.wieczorek86@gmail.com</t>
+          <t>wojciech.wieczorek86@interia.pl</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
@@ -7933,7 +7933,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>justyna.jablonska@nova-data.pl</t>
+          <t>justyna.jablonska@o2.pl</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
@@ -8025,7 +8025,7 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>p.witkowski@biuro.pl</t>
+          <t>p.witkowski@domena..pl</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -8117,7 +8117,7 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>walczak.maria@poczta.pl</t>
+          <t>walczak.maria@outlook.com</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -8209,7 +8209,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>michalstepien@mail.pl</t>
+          <t>michalstepien@yahoo.com</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>joanna_baran@silesia-invest.pl</t>
+          <t>joanna_baran@icloud.com</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -8393,7 +8393,7 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>pawel.rutkowski92@wp.pl</t>
+          <t>pawel.rutkowski92@gmail.com</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
@@ -8485,7 +8485,7 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>magdalena.gorska@gmail.com</t>
+          <t>magdalena.gorska@.pl</t>
         </is>
       </c>
       <c r="R92" t="inlineStr">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>r.sikora@proton.me</t>
+          <t>r.sikora@onet.pl</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
@@ -8669,7 +8669,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>ostrowska.agnieszka@helios-markets.pl</t>
+          <t>ostrowska.agnieszka@interia.pl</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>wojciechtomaszewski@poczta.pl</t>
+          <t>wojciechtomaszewski@o2.pl</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
@@ -8853,7 +8853,7 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>justyna_zajac@mail.pl</t>
+          <t>justyna_zajac@proton.me</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">
@@ -8945,7 +8945,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>piotr.pietrzak98@onet.pl</t>
+          <t>piotr.pietrzak98@domena..pl</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -9037,7 +9037,7 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>maria.wojcicka@polaris-capital.pl</t>
+          <t>maria.wojcicka@yahoo.com</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>m.czarnecki@gmail.com</t>
+          <t>m.czarnecki@icloud.com</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
@@ -9221,7 +9221,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>lis.joanna@proton.me</t>
+          <t>lis.joanna@gmail.com</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -9313,7 +9313,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>pawelkolodziej@biuro.pl</t>
+          <t>pawelkolodziej@wp.pl</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -9405,7 +9405,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>magdalena_kaczmarek@astra-finance.pl</t>
+          <t>magdalena_kaczmarek@.pl</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -9497,7 +9497,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>robert.piatek75@mail.pl</t>
+          <t>robert.piatek75@interia.pl</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -9589,7 +9589,7 @@
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>agnieszka.sadowska@onet.pl</t>
+          <t>agnieszka.sadowska@o2.pl</t>
         </is>
       </c>
       <c r="R104" t="inlineStr">
@@ -9681,7 +9681,7 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>w.wlodarczyk@wp.pl</t>
+          <t>w.wlodarczyk@proton.me</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
@@ -9773,7 +9773,7 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>borkowska.justyna@nova-data.pl</t>
+          <t>borkowska.justyna@outlook.com</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
@@ -9865,7 +9865,7 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>piotrkowalski@proton.me</t>
+          <t>piotrkowalski@domena..pl</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -9957,7 +9957,7 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>maria_nowacka@biuro.pl</t>
+          <t>maria_nowacka@icloud.com</t>
         </is>
       </c>
       <c r="R108" t="inlineStr">
@@ -10049,7 +10049,7 @@
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>michal.wisniewski81@poczta.pl</t>
+          <t>michal.wisniewski81@gmail.com</t>
         </is>
       </c>
       <c r="R109" t="inlineStr">
@@ -10141,7 +10141,7 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>joanna.wojcik@silesia-invest.pl</t>
+          <t>joanna.wojcik@wp.pl</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
@@ -10325,7 +10325,7 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>kaminska.magdalena@wp.pl</t>
+          <t>kaminska.magdalena@.pl</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -10417,7 +10417,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>robertlewandowski@gmail.com</t>
+          <t>robertlewandowski@o2.pl</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>agnieszka_zielinska@helios-markets.pl</t>
+          <t>agnieszka_zielinska@proton.me</t>
         </is>
       </c>
       <c r="R114" t="inlineStr">
@@ -10601,7 +10601,7 @@
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>wojciech.szymanski87@biuro.pl</t>
+          <t>wojciech.szymanski87@outlook.com</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -10693,7 +10693,7 @@
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>justyna.dabrowska@poczta.pl</t>
+          <t>justyna.dabrowska@yahoo.com</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -10785,7 +10785,7 @@
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>p.mazur@mail.pl</t>
+          <t>p.mazur@domena..pl</t>
         </is>
       </c>
       <c r="R117" t="inlineStr">
@@ -10877,7 +10877,7 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>krawczyk.maria@polaris-capital.pl</t>
+          <t>krawczyk.maria@gmail.com</t>
         </is>
       </c>
       <c r="R118" t="inlineStr">
@@ -11061,7 +11061,7 @@
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>joanna_jankowska@gmail.com</t>
+          <t>joanna_jankowska@onet.pl</t>
         </is>
       </c>
       <c r="R120" t="inlineStr">
@@ -11153,7 +11153,7 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>pawel.grabowski93@proton.me</t>
+          <t>pawel.grabowski93@interia.pl</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
@@ -11245,7 +11245,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>magdalena.pawlak@astra-finance.pl</t>
+          <t>magdalena.pawlak@.pl</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
@@ -11337,7 +11337,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>r.michalski@poczta.pl</t>
+          <t>r.michalski@proton.me</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
@@ -11429,7 +11429,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>krol.agnieszka@mail.pl</t>
+          <t>krol.agnieszka@outlook.com</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
@@ -11521,7 +11521,7 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>wojciechwieczorek@onet.pl</t>
+          <t>wojciechwieczorek@yahoo.com</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
@@ -11613,7 +11613,7 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>justyna_jablonska@nova-data.pl</t>
+          <t>justyna_jablonska@icloud.com</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
@@ -11705,7 +11705,7 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>piotr.witkowski70@gmail.com</t>
+          <t>piotr.witkowski70@domena..pl</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
@@ -11797,7 +11797,7 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>maria.walczak@proton.me</t>
+          <t>maria.walczak@wp.pl</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
@@ -11981,7 +11981,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>baran.joanna@silesia-invest.pl</t>
+          <t>baran.joanna@onet.pl</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
@@ -12073,7 +12073,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>pawelrutkowski@mail.pl</t>
+          <t>pawelrutkowski@interia.pl</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
@@ -12165,7 +12165,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>magdalena_gorska@onet.pl</t>
+          <t>magdalena_gorska@o2.pl</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -12257,7 +12257,7 @@
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>robert.sikora76@wp.pl</t>
+          <t>robert.sikora76@.pl</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
@@ -12349,7 +12349,7 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>agnieszka.ostrowska@helios-markets.pl</t>
+          <t>agnieszka.ostrowska@outlook.com</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
@@ -12441,7 +12441,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>w.tomaszewski@proton.me</t>
+          <t>w.tomaszewski@yahoo.com</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -12533,7 +12533,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>zajac.justyna@biuro.pl</t>
+          <t>zajac.justyna@icloud.com</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
@@ -12625,7 +12625,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>piotrpietrzak@poczta.pl</t>
+          <t>piotrpietrzak@gmail.com</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -12717,7 +12717,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>maria_wojcicka@polaris-capital.pl</t>
+          <t>maria_wojcicka@domena..pl</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
@@ -12901,7 +12901,7 @@
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>joanna.lis@wp.pl</t>
+          <t>joanna.lis@interia.pl</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
@@ -12993,7 +12993,7 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>p.kolodziej@gmail.com</t>
+          <t>p.kolodziej@o2.pl</t>
         </is>
       </c>
       <c r="R141" t="inlineStr">
@@ -13085,7 +13085,7 @@
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>kaczmarek.magdalena@astra-finance.pl</t>
+          <t>kaczmarek.magdalena@proton.me</t>
         </is>
       </c>
       <c r="R142" t="inlineStr">
@@ -13177,7 +13177,7 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>robertpiatek@biuro.pl</t>
+          <t>robertpiatek@.pl</t>
         </is>
       </c>
       <c r="R143" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>agnieszka_sadowska@poczta.pl</t>
+          <t>agnieszka_sadowska@yahoo.com</t>
         </is>
       </c>
       <c r="R144" t="inlineStr">
@@ -13361,7 +13361,7 @@
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>wojciech.wlodarczyk88@mail.pl</t>
+          <t>wojciech.wlodarczyk88@icloud.com</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
@@ -13453,7 +13453,7 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>justyna.borkowska@nova-data.pl</t>
+          <t>justyna.borkowska@gmail.com</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
@@ -13637,7 +13637,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>nowacka.maria@gmail.com</t>
+          <t>nowacka.maria@domena..pl</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
@@ -13729,7 +13729,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>michalwisniewski@proton.me</t>
+          <t>michalwisniewski@interia.pl</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
@@ -13821,7 +13821,7 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>joanna_wojcik@silesia-invest.pl</t>
+          <t>joanna_wojcik@o2.pl</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
@@ -13913,7 +13913,7 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>pawel.kowalczyk94@poczta.pl</t>
+          <t>pawel.kowalczyk94@proton.me</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
@@ -14005,7 +14005,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>magdalena.kaminska@mail.pl</t>
+          <t>magdalena.kaminska@outlook.com</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
@@ -14097,7 +14097,7 @@
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>r.lewandowski@onet.pl</t>
+          <t>r.lewandowski@yahoo.com</t>
         </is>
       </c>
       <c r="R153" t="inlineStr">
@@ -14189,7 +14189,7 @@
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>zielinska.agnieszka@helios-markets.pl</t>
+          <t>zielinska.agnieszka@wp</t>
         </is>
       </c>
       <c r="R154" t="inlineStr">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>justyna_dabrowska@proton.me</t>
+          <t>justyna_dabrowska@wp.pl</t>
         </is>
       </c>
       <c r="R156" t="inlineStr">
@@ -14465,7 +14465,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>piotr.mazur71@biuro.pl</t>
+          <t>piotr.mazur71@onet.pl</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
@@ -14557,7 +14557,7 @@
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>maria.krawczyk@polaris-capital.pl</t>
+          <t>maria.krawczyk@interia.pl</t>
         </is>
       </c>
       <c r="R158" t="inlineStr">
@@ -14649,7 +14649,7 @@
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>m.wozniak@mail.pl</t>
+          <t>@m.wozniak.invalid</t>
         </is>
       </c>
       <c r="R159" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>jankowska.joanna@onet.pl</t>
+          <t>jankowska.joanna@proton.me</t>
         </is>
       </c>
       <c r="R160" t="inlineStr">
@@ -14833,7 +14833,7 @@
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>pawelgrabowski@wp.pl</t>
+          <t>pawelgrabowski@outlook.com</t>
         </is>
       </c>
       <c r="R161" t="inlineStr">
@@ -14925,7 +14925,7 @@
       </c>
       <c r="Q162" t="inlineStr">
         <is>
-          <t>magdalena_pawlak@astra-finance.pl</t>
+          <t>magdalena_pawlak@yahoo.com</t>
         </is>
       </c>
       <c r="R162" t="inlineStr">
@@ -15017,7 +15017,7 @@
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>robert.michalski77@proton.me</t>
+          <t>robert.michalski77@icloud.com</t>
         </is>
       </c>
       <c r="R163" t="inlineStr">
@@ -15109,7 +15109,7 @@
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>agnieszka.krol@biuro.pl</t>
+          <t>agnieszka.krol@wp</t>
         </is>
       </c>
       <c r="R164" t="inlineStr">
@@ -15201,7 +15201,7 @@
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>w.wieczorek@poczta.pl</t>
+          <t>w.wieczorek@wp.pl</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
@@ -15293,7 +15293,7 @@
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>jablonska.justyna@nova-data.pl</t>
+          <t>jablonska.justyna@onet.pl</t>
         </is>
       </c>
       <c r="R166" t="inlineStr">
@@ -15385,7 +15385,7 @@
       </c>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>piotrwitkowski@onet.pl</t>
+          <t>piotrwitkowski@interia.pl</t>
         </is>
       </c>
       <c r="R167" t="inlineStr">
@@ -15477,7 +15477,7 @@
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>maria_walczak@wp.pl</t>
+          <t>maria_walczak@o2.pl</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
@@ -15569,7 +15569,7 @@
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>michal.stepien83@gmail.com</t>
+          <t>@michal.stepien83.invalid</t>
         </is>
       </c>
       <c r="R169" t="inlineStr">
@@ -15661,7 +15661,7 @@
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>joanna.baran@silesia-invest.pl</t>
+          <t>joanna.baran@outlook.com</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
@@ -15753,7 +15753,7 @@
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>p.rutkowski@biuro.pl</t>
+          <t>p.rutkowski@yahoo.com</t>
         </is>
       </c>
       <c r="R171" t="inlineStr">
@@ -15845,7 +15845,7 @@
       </c>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>gorska.magdalena@poczta.pl</t>
+          <t>gorska.magdalena@icloud.com</t>
         </is>
       </c>
       <c r="R172" t="inlineStr">
@@ -15937,7 +15937,7 @@
       </c>
       <c r="Q173" t="inlineStr">
         <is>
-          <t>robertsikora@mail.pl</t>
+          <t>robertsikora@gmail.com</t>
         </is>
       </c>
       <c r="R173" t="inlineStr">
@@ -16029,7 +16029,7 @@
       </c>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>agnieszka_ostrowska@helios-markets.pl</t>
+          <t>agnieszka_ostrowska@wp</t>
         </is>
       </c>
       <c r="R174" t="inlineStr">
@@ -16121,7 +16121,7 @@
       </c>
       <c r="Q175" t="inlineStr">
         <is>
-          <t>wojciech.tomaszewski89@wp.pl</t>
+          <t>wojciech.tomaszewski89@onet.pl</t>
         </is>
       </c>
       <c r="R175" t="inlineStr">
@@ -16213,7 +16213,7 @@
       </c>
       <c r="Q176" t="inlineStr">
         <is>
-          <t>justyna.zajac@gmail.com</t>
+          <t>justyna.zajac@interia.pl</t>
         </is>
       </c>
       <c r="R176" t="inlineStr">
@@ -16305,7 +16305,7 @@
       </c>
       <c r="Q177" t="inlineStr">
         <is>
-          <t>p.pietrzak@proton.me</t>
+          <t>p.pietrzak@o2.pl</t>
         </is>
       </c>
       <c r="R177" t="inlineStr">
@@ -16397,7 +16397,7 @@
       </c>
       <c r="Q178" t="inlineStr">
         <is>
-          <t>wojcicka.maria@polaris-capital.pl</t>
+          <t>wojcicka.maria@proton.me</t>
         </is>
       </c>
       <c r="R178" t="inlineStr">
@@ -16489,7 +16489,7 @@
       </c>
       <c r="Q179" t="inlineStr">
         <is>
-          <t>michalczarnecki@poczta.pl</t>
+          <t>@michalczarnecki.invalid</t>
         </is>
       </c>
       <c r="R179" t="inlineStr">
@@ -16581,7 +16581,7 @@
       </c>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>joanna_lis@mail.pl</t>
+          <t>joanna_lis@yahoo.com</t>
         </is>
       </c>
       <c r="R180" t="inlineStr">
@@ -16673,7 +16673,7 @@
       </c>
       <c r="Q181" t="inlineStr">
         <is>
-          <t>pawel.kolodziej95@onet.pl</t>
+          <t>pawel.kolodziej95@icloud.com</t>
         </is>
       </c>
       <c r="R181" t="inlineStr">
@@ -16765,7 +16765,7 @@
       </c>
       <c r="Q182" t="inlineStr">
         <is>
-          <t>magdalena.kaczmarek@astra-finance.pl</t>
+          <t>magdalena.kaczmarek@gmail.com</t>
         </is>
       </c>
       <c r="R182" t="inlineStr">
@@ -16857,7 +16857,7 @@
       </c>
       <c r="Q183" t="inlineStr">
         <is>
-          <t>r.piatek@gmail.com</t>
+          <t>r.piatek@wp.pl</t>
         </is>
       </c>
       <c r="R183" t="inlineStr">
@@ -16949,7 +16949,7 @@
       </c>
       <c r="Q184" t="inlineStr">
         <is>
-          <t>sadowska.agnieszka@proton.me</t>
+          <t>sadowska.agnieszka@wp</t>
         </is>
       </c>
       <c r="R184" t="inlineStr">
@@ -17041,7 +17041,7 @@
       </c>
       <c r="Q185" t="inlineStr">
         <is>
-          <t>wojciechwlodarczyk@biuro.pl</t>
+          <t>wojciechwlodarczyk@interia.pl</t>
         </is>
       </c>
       <c r="R185" t="inlineStr">
@@ -17133,7 +17133,7 @@
       </c>
       <c r="Q186" t="inlineStr">
         <is>
-          <t>justyna_borkowska@nova-data.pl</t>
+          <t>justyna_borkowska@o2.pl</t>
         </is>
       </c>
       <c r="R186" t="inlineStr">
@@ -17225,7 +17225,7 @@
       </c>
       <c r="Q187" t="inlineStr">
         <is>
-          <t>piotr.kowalski72@mail.pl</t>
+          <t>piotr.kowalski72@proton.me</t>
         </is>
       </c>
       <c r="R187" t="inlineStr">
@@ -17317,7 +17317,7 @@
       </c>
       <c r="Q188" t="inlineStr">
         <is>
-          <t>maria.nowacka@onet.pl</t>
+          <t>maria.nowacka@outlook.com</t>
         </is>
       </c>
       <c r="R188" t="inlineStr">
@@ -17409,7 +17409,7 @@
       </c>
       <c r="Q189" t="inlineStr">
         <is>
-          <t>m.wisniewski@wp.pl</t>
+          <t>@m.wisniewski.invalid</t>
         </is>
       </c>
       <c r="R189" t="inlineStr">
@@ -17501,7 +17501,7 @@
       </c>
       <c r="Q190" t="inlineStr">
         <is>
-          <t>wojcik.joanna@silesia-invest.pl</t>
+          <t>wojcik.joanna@icloud.com</t>
         </is>
       </c>
       <c r="R190" t="inlineStr">
@@ -17593,7 +17593,7 @@
       </c>
       <c r="Q191" t="inlineStr">
         <is>
-          <t>pawelkowalczyk@proton.me</t>
+          <t>pawelkowalczyk@gmail.com</t>
         </is>
       </c>
       <c r="R191" t="inlineStr">
@@ -17685,7 +17685,7 @@
       </c>
       <c r="Q192" t="inlineStr">
         <is>
-          <t>magdalena_kaminska@biuro.pl</t>
+          <t>magdalena_kaminska@wp.pl</t>
         </is>
       </c>
       <c r="R192" t="inlineStr">
@@ -17777,7 +17777,7 @@
       </c>
       <c r="Q193" t="inlineStr">
         <is>
-          <t>robert.lewandowski78@poczta.pl</t>
+          <t>robert.lewandowski78@onet.pl</t>
         </is>
       </c>
       <c r="R193" t="inlineStr">
@@ -17869,7 +17869,7 @@
       </c>
       <c r="Q194" t="inlineStr">
         <is>
-          <t>agnieszka.zielinska@helios-markets.pl</t>
+          <t>agnieszka.zielinska@wp</t>
         </is>
       </c>
       <c r="R194" t="inlineStr">
@@ -17961,7 +17961,7 @@
       </c>
       <c r="Q195" t="inlineStr">
         <is>
-          <t>w.szymanski@onet.pl</t>
+          <t>w.szymanski@o2.pl</t>
         </is>
       </c>
       <c r="R195" t="inlineStr">
@@ -18053,7 +18053,7 @@
       </c>
       <c r="Q196" t="inlineStr">
         <is>
-          <t>dabrowska.justyna@wp.pl</t>
+          <t>dabrowska.justyna@proton.me</t>
         </is>
       </c>
       <c r="R196" t="inlineStr">
@@ -18145,7 +18145,7 @@
       </c>
       <c r="Q197" t="inlineStr">
         <is>
-          <t>piotrmazur@gmail.com</t>
+          <t>piotrmazur@outlook.com</t>
         </is>
       </c>
       <c r="R197" t="inlineStr">
@@ -18237,7 +18237,7 @@
       </c>
       <c r="Q198" t="inlineStr">
         <is>
-          <t>maria_krawczyk@polaris-capital.pl</t>
+          <t>maria_krawczyk@yahoo.com</t>
         </is>
       </c>
       <c r="R198" t="inlineStr">
@@ -18329,7 +18329,7 @@
       </c>
       <c r="Q199" t="inlineStr">
         <is>
-          <t>michal.wozniak84@biuro.pl</t>
+          <t>@michal.wozniak84.invalid</t>
         </is>
       </c>
       <c r="R199" t="inlineStr">
@@ -18421,7 +18421,7 @@
       </c>
       <c r="Q200" t="inlineStr">
         <is>
-          <t>joanna.jankowska@poczta.pl</t>
+          <t>joanna.jankowska@gmail.com</t>
         </is>
       </c>
       <c r="R200" t="inlineStr">
@@ -18513,7 +18513,7 @@
       </c>
       <c r="Q201" t="inlineStr">
         <is>
-          <t>p.grabowski@mail.pl</t>
+          <t>p.grabowski@wp.pl</t>
         </is>
       </c>
       <c r="R201" t="inlineStr">

</xml_diff>

<commit_message>
Zwiekszenie liczby poprawnych maili
</commit_message>
<xml_diff>
--- a/data/xlsx/ceidg.xlsx
+++ b/data/xlsx/ceidg.xlsx
@@ -205,7 +205,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>magdalena.pawlak@interia.pl</t>
+          <t>magdalena.pawlak@tmp.ii</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -297,7 +297,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>r.michalski@o2.pl</t>
+          <t>r.michalski@foo.zz</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -389,7 +389,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>krol.agnieszka@brak-domeny</t>
+          <t>krol.agnieszka@bar.yy</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -481,7 +481,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>wojciechwieczorek@outlook.com</t>
+          <t>wojciechwieczorek@zzz.uu</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>justyna_jablonska@yahoo.com</t>
+          <t>justyna_jablonska@uuu.ii</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>piotr.witkowski95@icloud.com</t>
+          <t>piotr.witkowski95@qqq.zz</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>maria.walczak@gmail.com</t>
+          <t>maria.walczak@abc.yy</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>m.stepien@localhost</t>
+          <t>m.stepien@xxx.uu</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>baran.joanna@onet.pl</t>
+          <t>baran.joanna@interia.pl</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>pawelrutkowski@interia.pl</t>
+          <t>pawelrutkowski@o2.pl</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>magdalena_gorska@o2.pl</t>
+          <t>magdalena_gorska@proton.me</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>robert.sikora72@proton.me</t>
+          <t>robert.sikora72@outlook.com</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>agnieszka.ostrowska@brak-domeny</t>
+          <t>agnieszka.ostrowska@yahoo.com</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>w.tomaszewski@yahoo.com</t>
+          <t>w.tomaszewski@icloud.com</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>zajac.justyna@icloud.com</t>
+          <t>zajac.justyna@gmail.com</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>piotrpietrzak@gmail.com</t>
+          <t>piotrpietrzak@wp.pl</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>maria_wojcicka@wp.pl</t>
+          <t>maria_wojcicka@onet.pl</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>michal.czarnecki78@localhost</t>
+          <t>michal.czarnecki78@interia.pl</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>joanna.lis@interia.pl</t>
+          <t>joanna.lis@o2.pl</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>p.kolodziej@o2.pl</t>
+          <t>p.kolodziej@proton.me</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>kaczmarek.magdalena@proton.me</t>
+          <t>kaczmarek.magdalena@outlook.com</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>robertpiatek@outlook.com</t>
+          <t>robertpiatek@yahoo.com</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>agnieszka_sadowska@brak-domeny</t>
+          <t>agnieszka_sadowska@icloud.com</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>wojciech.wlodarczyk84@icloud.com</t>
+          <t>wojciech.wlodarczyk84@gmail.com</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>justyna.borkowska@gmail.com</t>
+          <t>justyna.borkowska@wp.pl</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>p.kowalski@wp.pl</t>
+          <t>p.kowalski@onet.pl</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>nowacka.maria@onet.pl</t>
+          <t>nowacka.maria@interia.pl</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>michalwisniewski@gmailcom</t>
+          <t>michalwisniewski@o2.pl</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>joanna_wojcik@localhost</t>
+          <t>joanna_wojcik@proton.me</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>pawel.kowalczyk90@o2.pl</t>
+          <t>pawel.kowalczyk90@outlook.com</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>magdalena.kaminska@proton.me</t>
+          <t>magdalena.kaminska@yahoo.com</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>r.lewandowski@outlook.com</t>
+          <t>r.lewandowski@icloud.com</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3149,7 +3149,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>zielinska.agnieszka@yahoo.com</t>
+          <t>zielinska.agnieszka@gmail.com</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>wojciechszymanski@brak-domeny</t>
+          <t>wojciechszymanski@wp.pl</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>justyna_dabrowska@gmail.com</t>
+          <t>justyna_dabrowska@onet.pl</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>piotr.mazur96@wp.pl</t>
+          <t>piotr.mazur96@interia.pl</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>maria.krawczyk@onet.pl</t>
+          <t>maria.krawczyk@o2.pl</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>m.wozniak@interia.pl</t>
+          <t>m.wozniak@proton.me</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>jankowska.joanna@localhost</t>
+          <t>jankowska.joanna@outlook.com</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>pawelgrabowski@proton.me</t>
+          <t>pawelgrabowski@yahoo.com</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>magdalena_pawlak@outlook.com</t>
+          <t>magdalena_pawlak@icloud.com</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -3977,7 +3977,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>robert.michalski73@yahoo.com</t>
+          <t>robert.michalski73@gmail.com</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>agnieszka.krol@icloud.com</t>
+          <t>agnieszka.krol@wp.pl</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>w.wieczorek@brak-domeny</t>
+          <t>w.wieczorek@onet.pl</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>jablonska.justyna@wp.pl</t>
+          <t>jablonska.justyna@interia.pl</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4345,7 +4345,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>piotrwitkowski@onet.pl</t>
+          <t>piotrwitkowski@o2.pl</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4437,7 +4437,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>maria_walczak@interia.pl</t>
+          <t>maria_walczak@proton.me</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -4529,7 +4529,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>michal.stepien79@o2.pl</t>
+          <t>michal.stepien79@outlook.com</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4621,7 +4621,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>joanna.baran@localhost</t>
+          <t>joanna.baran@yahoo.com</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>p.rutkowski@outlook.com</t>
+          <t>p.rutkowski@icloud.com</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>gorska.magdalena@yahoo.com</t>
+          <t>gorska.magdalena@gmail.com</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>robertsikora@icloud.com</t>
+          <t>robertsikora@wp.pl</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>agnieszka_ostrowska@gmail.com</t>
+          <t>agnieszka_ostrowska@onet.pl</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>wojciech.tomaszewski85@wp.pl</t>
+          <t>wojciech.tomaszewski85@interia.pl</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5173,7 +5173,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>justyna.zajac@domena..pl</t>
+          <t>justyna.zajac@o2.pl</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>p.pietrzak@interia.pl</t>
+          <t>p.pietrzak@proton.me</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5357,7 +5357,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>wojcicka.maria@o2.pl</t>
+          <t>wojcicka.maria@outlook.com</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5449,7 +5449,7 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>michalczarnecki@proton.me</t>
+          <t>michalczarnecki@yahoo.com</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -5541,7 +5541,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>joanna_lis@outlook.com</t>
+          <t>joanna_lis@icloud.com</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>pawel.kolodziej91@.pl</t>
+          <t>pawel.kolodziej91@gmail.com</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -5725,7 +5725,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>magdalena.kaczmarek@icloud.com</t>
+          <t>magdalena.kaczmarek@wp.pl</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -5817,7 +5817,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>r.piatek@gmail.com</t>
+          <t>r.piatek@onet.pl</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -5909,7 +5909,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>sadowska.agnieszka@wp.pl</t>
+          <t>sadowska.agnieszka@interia.pl</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -6001,7 +6001,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>wojciechwlodarczyk@onet.pl</t>
+          <t>wojciechwlodarczyk@o2.pl</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -6093,7 +6093,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>justyna_borkowska@domena..pl</t>
+          <t>justyna_borkowska@proton.me</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -6185,7 +6185,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>piotr.kowalski97@o2.pl</t>
+          <t>piotr.kowalski97@outlook.com</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -6277,7 +6277,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>maria.nowacka@proton.me</t>
+          <t>maria.nowacka@yahoo.com</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -6369,7 +6369,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>m.wisniewski@outlook.com</t>
+          <t>m.wisniewski@icloud.com</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
@@ -6461,7 +6461,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>wojcik.joanna@yahoo.com</t>
+          <t>wojcik.joanna@gmail.com</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>pawelkowalczyk@.pl</t>
+          <t>pawelkowalczyk@wp.pl</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -6645,7 +6645,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>magdalena_kaminska@gmail.com</t>
+          <t>magdalena_kaminska@onet.pl</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -6737,7 +6737,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>robert.lewandowski74@wp.pl</t>
+          <t>robert.lewandowski74@interia.pl</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -6829,7 +6829,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>agnieszka.zielinska@onet.pl</t>
+          <t>agnieszka.zielinska@o2.pl</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>w.szymanski@interia.pl</t>
+          <t>w.szymanski@proton.me</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -7013,7 +7013,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>dabrowska.justyna@domena..pl</t>
+          <t>dabrowska.justyna@outlook.com</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -7105,7 +7105,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>piotrmazur@proton.me</t>
+          <t>piotrmazur@yahoo.com</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -7197,7 +7197,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>maria_krawczyk@outlook.com</t>
+          <t>maria_krawczyk@icloud.com</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -7289,7 +7289,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>michal.wozniak80@yahoo.com</t>
+          <t>michal.wozniak80@gmail.com</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -7381,7 +7381,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>joanna.jankowska@icloud.com</t>
+          <t>joanna.jankowska@wp.pl</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -7473,7 +7473,7 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>p.grabowski@.pl</t>
+          <t>p.grabowski@onet.pl</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -7565,7 +7565,7 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>pawlak.magdalena@wp.pl</t>
+          <t>pawlak.magdalena@interia.pl</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -7657,7 +7657,7 @@
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>robertmichalski@onet.pl</t>
+          <t>robertmichalski@o2.pl</t>
         </is>
       </c>
       <c r="R83" t="inlineStr">
@@ -7841,7 +7841,7 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>wojciech.wieczorek86@interia.pl</t>
+          <t>wojciech.wieczorek86@proton.me</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
@@ -7933,7 +7933,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>justyna.jablonska@o2.pl</t>
+          <t>justyna.jablonska@outlook.com</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
@@ -8025,7 +8025,7 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>p.witkowski@domena..pl</t>
+          <t>p.witkowski@yahoo.com</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -8117,7 +8117,7 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>walczak.maria@outlook.com</t>
+          <t>walczak.maria@icloud.com</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -8209,7 +8209,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>michalstepien@yahoo.com</t>
+          <t>michalstepien@gmail.com</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>joanna_baran@icloud.com</t>
+          <t>joanna_baran@wp.pl</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -8393,7 +8393,7 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>pawel.rutkowski92@gmail.com</t>
+          <t>pawel.rutkowski92@onet.pl</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
@@ -8485,7 +8485,7 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>magdalena.gorska@.pl</t>
+          <t>magdalena.gorska@interia.pl</t>
         </is>
       </c>
       <c r="R92" t="inlineStr">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>r.sikora@onet.pl</t>
+          <t>r.sikora@o2.pl</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
@@ -8669,7 +8669,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>ostrowska.agnieszka@interia.pl</t>
+          <t>ostrowska.agnieszka@proton.me</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>wojciechtomaszewski@o2.pl</t>
+          <t>wojciechtomaszewski@outlook.com</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
@@ -8853,7 +8853,7 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>justyna_zajac@proton.me</t>
+          <t>justyna_zajac@yahoo.com</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">
@@ -8945,7 +8945,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>piotr.pietrzak98@domena..pl</t>
+          <t>piotr.pietrzak98@icloud.com</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -9037,7 +9037,7 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>maria.wojcicka@yahoo.com</t>
+          <t>maria.wojcicka@gmail.com</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>m.czarnecki@icloud.com</t>
+          <t>m.czarnecki@wp.pl</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
@@ -9221,7 +9221,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>lis.joanna@gmail.com</t>
+          <t>lis.joanna@onet.pl</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -9313,7 +9313,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>pawelkolodziej@wp.pl</t>
+          <t>pawelkolodziej@interia.pl</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -9405,7 +9405,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>magdalena_kaczmarek@.pl</t>
+          <t>magdalena_kaczmarek@o2.pl</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -9497,7 +9497,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>robert.piatek75@interia.pl</t>
+          <t>robert.piatek75@qqq.zz</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -9589,7 +9589,7 @@
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>agnieszka.sadowska@o2.pl</t>
+          <t>agnieszka.sadowska@abc.yy</t>
         </is>
       </c>
       <c r="R104" t="inlineStr">
@@ -9681,7 +9681,7 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>w.wlodarczyk@proton.me</t>
+          <t>w.wlodarczyk@xxx.uu</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
@@ -9773,7 +9773,7 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>borkowska.justyna@outlook.com</t>
+          <t>borkowska.justyna@bbb.ii</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
@@ -9865,7 +9865,7 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>piotrkowalski@domena..pl</t>
+          <t>piotrkowalski@mmm.zz</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -9957,7 +9957,7 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>maria_nowacka@icloud.com</t>
+          <t>maria_nowacka@nnn.yy</t>
         </is>
       </c>
       <c r="R108" t="inlineStr">
@@ -10049,7 +10049,7 @@
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>michal.wisniewski81@gmail.com</t>
+          <t>michal.wisniewski81@kkk.uu</t>
         </is>
       </c>
       <c r="R109" t="inlineStr">
@@ -10141,7 +10141,7 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>joanna.wojcik@wp.pl</t>
+          <t>joanna.wojcik@tmp.ii</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>p.kowalczyk@onet.pl</t>
+          <t>p.kowalczyk@o2.pl</t>
         </is>
       </c>
       <c r="R111" t="inlineStr">
@@ -10325,7 +10325,7 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>kaminska.magdalena@.pl</t>
+          <t>kaminska.magdalena@proton.me</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -10417,7 +10417,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>robertlewandowski@o2.pl</t>
+          <t>robertlewandowski@outlook.com</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>agnieszka_zielinska@proton.me</t>
+          <t>agnieszka_zielinska@yahoo.com</t>
         </is>
       </c>
       <c r="R114" t="inlineStr">
@@ -10601,7 +10601,7 @@
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>wojciech.szymanski87@outlook.com</t>
+          <t>wojciech.szymanski87@icloud.com</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -10693,7 +10693,7 @@
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>justyna.dabrowska@yahoo.com</t>
+          <t>justyna.dabrowska@gmail.com</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -10785,7 +10785,7 @@
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>p.mazur@domena..pl</t>
+          <t>p.mazur@wp.pl</t>
         </is>
       </c>
       <c r="R117" t="inlineStr">
@@ -10877,7 +10877,7 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>krawczyk.maria@gmail.com</t>
+          <t>krawczyk.maria@onet.pl</t>
         </is>
       </c>
       <c r="R118" t="inlineStr">
@@ -10969,7 +10969,7 @@
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>michalwozniak@wp.pl</t>
+          <t>michalwozniak@interia.pl</t>
         </is>
       </c>
       <c r="R119" t="inlineStr">
@@ -11061,7 +11061,7 @@
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>joanna_jankowska@onet.pl</t>
+          <t>joanna_jankowska@o2.pl</t>
         </is>
       </c>
       <c r="R120" t="inlineStr">
@@ -11153,7 +11153,7 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>pawel.grabowski93@interia.pl</t>
+          <t>pawel.grabowski93@proton.me</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
@@ -11245,7 +11245,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>magdalena.pawlak@.pl</t>
+          <t>magdalena.pawlak@outlook.com</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
@@ -11337,7 +11337,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>r.michalski@proton.me</t>
+          <t>r.michalski@yahoo.com</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
@@ -11429,7 +11429,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>krol.agnieszka@outlook.com</t>
+          <t>krol.agnieszka@icloud.com</t>
         </is>
       </c>
       <c r="R124" t="inlineStr">
@@ -11521,7 +11521,7 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>wojciechwieczorek@yahoo.com</t>
+          <t>wojciechwieczorek@gmail.com</t>
         </is>
       </c>
       <c r="R125" t="inlineStr">
@@ -11613,7 +11613,7 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>justyna_jablonska@icloud.com</t>
+          <t>justyna_jablonska@wp.pl</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
@@ -11705,7 +11705,7 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>piotr.witkowski70@domena..pl</t>
+          <t>piotr.witkowski70@onet.pl</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
@@ -11797,7 +11797,7 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>maria.walczak@wp.pl</t>
+          <t>maria.walczak@interia.pl</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
@@ -11889,7 +11889,7 @@
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>m.stepienbiuro.pl</t>
+          <t>m.stepienbiuro.pl@o2.pl</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
@@ -11981,7 +11981,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>baran.joanna@onet.pl</t>
+          <t>baran.joanna@proton.me</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
@@ -12073,7 +12073,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>pawelrutkowski@interia.pl</t>
+          <t>pawelrutkowski@outlook.com</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
@@ -12165,7 +12165,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>magdalena_gorska@o2.pl</t>
+          <t>magdalena_gorska@yahoo.com</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -12257,7 +12257,7 @@
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>robert.sikora76@.pl</t>
+          <t>robert.sikora76@icloud.com</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
@@ -12349,7 +12349,7 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>agnieszka.ostrowska@outlook.com</t>
+          <t>agnieszka.ostrowska@gmail.com</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
@@ -12441,7 +12441,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>w.tomaszewski@yahoo.com</t>
+          <t>w.tomaszewski@wp.pl</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -12533,7 +12533,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>zajac.justyna@icloud.com</t>
+          <t>zajac.justyna@onet.pl</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
@@ -12625,7 +12625,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>piotrpietrzak@gmail.com</t>
+          <t>piotrpietrzak@interia.pl</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -12717,7 +12717,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>maria_wojcicka@domena..pl</t>
+          <t>maria_wojcicka@o2.pl</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
@@ -12809,7 +12809,7 @@
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>michal.czarnecki82@onet.pl</t>
+          <t>michal.czarnecki82@proton.me</t>
         </is>
       </c>
       <c r="R139" t="inlineStr">
@@ -12901,7 +12901,7 @@
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>joanna.lis@interia.pl</t>
+          <t>joanna.lis@outlook.com</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
@@ -12993,7 +12993,7 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>p.kolodziej@o2.pl</t>
+          <t>p.kolodziej@yahoo.com</t>
         </is>
       </c>
       <c r="R141" t="inlineStr">
@@ -13085,7 +13085,7 @@
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>kaczmarek.magdalena@proton.me</t>
+          <t>kaczmarek.magdalena@icloud.com</t>
         </is>
       </c>
       <c r="R142" t="inlineStr">
@@ -13177,7 +13177,7 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>robertpiatek@.pl</t>
+          <t>robertpiatek@gmail.com</t>
         </is>
       </c>
       <c r="R143" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>agnieszka_sadowska@yahoo.com</t>
+          <t>agnieszka_sadowska@wp.pl</t>
         </is>
       </c>
       <c r="R144" t="inlineStr">
@@ -13361,7 +13361,7 @@
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>wojciech.wlodarczyk88@icloud.com</t>
+          <t>wojciech.wlodarczyk88@onet.pl</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
@@ -13453,7 +13453,7 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>justyna.borkowska@gmail.com</t>
+          <t>justyna.borkowska@interia.pl</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
@@ -13545,7 +13545,7 @@
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>p.kowalski@wp.pl</t>
+          <t>p.kowalski@o2.pl</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">
@@ -13637,7 +13637,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>nowacka.maria@domena..pl</t>
+          <t>nowacka.maria@proton.me</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
@@ -13729,7 +13729,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>michalwisniewski@interia.pl</t>
+          <t>michalwisniewski@outlook.com</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
@@ -13821,7 +13821,7 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>joanna_wojcik@o2.pl</t>
+          <t>joanna_wojcik@yahoo.com</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
@@ -13913,7 +13913,7 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>pawel.kowalczyk94@proton.me</t>
+          <t>pawel.kowalczyk94@icloud.com</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
@@ -14005,7 +14005,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>magdalena.kaminska@outlook.com</t>
+          <t>magdalena.kaminska@gmail.com</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
@@ -14097,7 +14097,7 @@
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>r.lewandowski@yahoo.com</t>
+          <t>r.lewandowski@wp.pl</t>
         </is>
       </c>
       <c r="R153" t="inlineStr">
@@ -14189,7 +14189,7 @@
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>zielinska.agnieszka@wp</t>
+          <t>zielinska.agnieszka@onet.pl</t>
         </is>
       </c>
       <c r="R154" t="inlineStr">
@@ -14281,7 +14281,7 @@
       </c>
       <c r="Q155" t="inlineStr">
         <is>
-          <t>wojciechszymanski@gmail.com</t>
+          <t>wojciechszymanski@interia.pl</t>
         </is>
       </c>
       <c r="R155" t="inlineStr">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>justyna_dabrowska@wp.pl</t>
+          <t>justyna_dabrowska@o2.pl</t>
         </is>
       </c>
       <c r="R156" t="inlineStr">
@@ -14465,7 +14465,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>piotr.mazur71@onet.pl</t>
+          <t>piotr.mazur71@proton.me</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
@@ -14557,7 +14557,7 @@
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>maria.krawczyk@interia.pl</t>
+          <t>maria.krawczyk@outlook.com</t>
         </is>
       </c>
       <c r="R158" t="inlineStr">
@@ -14649,7 +14649,7 @@
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>@m.wozniak.invalid</t>
+          <t>email.20740157@yahoo.com</t>
         </is>
       </c>
       <c r="R159" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>jankowska.joanna@proton.me</t>
+          <t>jankowska.joanna@icloud.com</t>
         </is>
       </c>
       <c r="R160" t="inlineStr">
@@ -14833,7 +14833,7 @@
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>pawelgrabowski@outlook.com</t>
+          <t>pawelgrabowski@gmail.com</t>
         </is>
       </c>
       <c r="R161" t="inlineStr">
@@ -14925,7 +14925,7 @@
       </c>
       <c r="Q162" t="inlineStr">
         <is>
-          <t>magdalena_pawlak@yahoo.com</t>
+          <t>magdalena_pawlak@wp.pl</t>
         </is>
       </c>
       <c r="R162" t="inlineStr">
@@ -15017,7 +15017,7 @@
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>robert.michalski77@icloud.com</t>
+          <t>robert.michalski77@onet.pl</t>
         </is>
       </c>
       <c r="R163" t="inlineStr">
@@ -15109,7 +15109,7 @@
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>agnieszka.krol@wp</t>
+          <t>agnieszka.krol@interia.pl</t>
         </is>
       </c>
       <c r="R164" t="inlineStr">
@@ -15201,7 +15201,7 @@
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>w.wieczorek@wp.pl</t>
+          <t>w.wieczorek@o2.pl</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
@@ -15293,7 +15293,7 @@
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>jablonska.justyna@onet.pl</t>
+          <t>jablonska.justyna@proton.me</t>
         </is>
       </c>
       <c r="R166" t="inlineStr">
@@ -15385,7 +15385,7 @@
       </c>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>piotrwitkowski@interia.pl</t>
+          <t>piotrwitkowski@outlook.com</t>
         </is>
       </c>
       <c r="R167" t="inlineStr">
@@ -15477,7 +15477,7 @@
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>maria_walczak@o2.pl</t>
+          <t>maria_walczak@yahoo.com</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
@@ -15569,7 +15569,7 @@
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>@michal.stepien83.invalid</t>
+          <t>email.20740167@icloud.com</t>
         </is>
       </c>
       <c r="R169" t="inlineStr">
@@ -15661,7 +15661,7 @@
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>joanna.baran@outlook.com</t>
+          <t>joanna.baran@gmail.com</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
@@ -15753,7 +15753,7 @@
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>p.rutkowski@yahoo.com</t>
+          <t>p.rutkowski@wp.pl</t>
         </is>
       </c>
       <c r="R171" t="inlineStr">
@@ -15845,7 +15845,7 @@
       </c>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>gorska.magdalena@icloud.com</t>
+          <t>gorska.magdalena@onet.pl</t>
         </is>
       </c>
       <c r="R172" t="inlineStr">
@@ -15937,7 +15937,7 @@
       </c>
       <c r="Q173" t="inlineStr">
         <is>
-          <t>robertsikora@gmail.com</t>
+          <t>robertsikora@interia.pl</t>
         </is>
       </c>
       <c r="R173" t="inlineStr">
@@ -16029,7 +16029,7 @@
       </c>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>agnieszka_ostrowska@wp</t>
+          <t>agnieszka_ostrowska@o2.pl</t>
         </is>
       </c>
       <c r="R174" t="inlineStr">
@@ -16121,7 +16121,7 @@
       </c>
       <c r="Q175" t="inlineStr">
         <is>
-          <t>wojciech.tomaszewski89@onet.pl</t>
+          <t>wojciech.tomaszewski89@proton.me</t>
         </is>
       </c>
       <c r="R175" t="inlineStr">
@@ -16213,7 +16213,7 @@
       </c>
       <c r="Q176" t="inlineStr">
         <is>
-          <t>justyna.zajac@interia.pl</t>
+          <t>justyna.zajac@outlook.com</t>
         </is>
       </c>
       <c r="R176" t="inlineStr">
@@ -16305,7 +16305,7 @@
       </c>
       <c r="Q177" t="inlineStr">
         <is>
-          <t>p.pietrzak@o2.pl</t>
+          <t>p.pietrzak@yahoo.com</t>
         </is>
       </c>
       <c r="R177" t="inlineStr">
@@ -16397,7 +16397,7 @@
       </c>
       <c r="Q178" t="inlineStr">
         <is>
-          <t>wojcicka.maria@proton.me</t>
+          <t>wojcicka.maria@icloud.com</t>
         </is>
       </c>
       <c r="R178" t="inlineStr">
@@ -16489,7 +16489,7 @@
       </c>
       <c r="Q179" t="inlineStr">
         <is>
-          <t>@michalczarnecki.invalid</t>
+          <t>email.20740177@gmail.com</t>
         </is>
       </c>
       <c r="R179" t="inlineStr">
@@ -16581,7 +16581,7 @@
       </c>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>joanna_lis@yahoo.com</t>
+          <t>joanna_lis@wp.pl</t>
         </is>
       </c>
       <c r="R180" t="inlineStr">
@@ -16673,7 +16673,7 @@
       </c>
       <c r="Q181" t="inlineStr">
         <is>
-          <t>pawel.kolodziej95@icloud.com</t>
+          <t>pawel.kolodziej95@onet.pl</t>
         </is>
       </c>
       <c r="R181" t="inlineStr">
@@ -16765,7 +16765,7 @@
       </c>
       <c r="Q182" t="inlineStr">
         <is>
-          <t>magdalena.kaczmarek@gmail.com</t>
+          <t>magdalena.kaczmarek@interia.pl</t>
         </is>
       </c>
       <c r="R182" t="inlineStr">
@@ -16857,7 +16857,7 @@
       </c>
       <c r="Q183" t="inlineStr">
         <is>
-          <t>r.piatek@wp.pl</t>
+          <t>r.piatek@o2.pl</t>
         </is>
       </c>
       <c r="R183" t="inlineStr">
@@ -16949,7 +16949,7 @@
       </c>
       <c r="Q184" t="inlineStr">
         <is>
-          <t>sadowska.agnieszka@wp</t>
+          <t>sadowska.agnieszka@proton.me</t>
         </is>
       </c>
       <c r="R184" t="inlineStr">
@@ -17041,7 +17041,7 @@
       </c>
       <c r="Q185" t="inlineStr">
         <is>
-          <t>wojciechwlodarczyk@interia.pl</t>
+          <t>wojciechwlodarczyk@outlook.com</t>
         </is>
       </c>
       <c r="R185" t="inlineStr">
@@ -17133,7 +17133,7 @@
       </c>
       <c r="Q186" t="inlineStr">
         <is>
-          <t>justyna_borkowska@o2.pl</t>
+          <t>justyna_borkowska@yahoo.com</t>
         </is>
       </c>
       <c r="R186" t="inlineStr">
@@ -17225,7 +17225,7 @@
       </c>
       <c r="Q187" t="inlineStr">
         <is>
-          <t>piotr.kowalski72@proton.me</t>
+          <t>piotr.kowalski72@icloud.com</t>
         </is>
       </c>
       <c r="R187" t="inlineStr">
@@ -17317,7 +17317,7 @@
       </c>
       <c r="Q188" t="inlineStr">
         <is>
-          <t>maria.nowacka@outlook.com</t>
+          <t>maria.nowacka@gmail.com</t>
         </is>
       </c>
       <c r="R188" t="inlineStr">
@@ -17409,7 +17409,7 @@
       </c>
       <c r="Q189" t="inlineStr">
         <is>
-          <t>@m.wisniewski.invalid</t>
+          <t>email.20740187@wp.pl</t>
         </is>
       </c>
       <c r="R189" t="inlineStr">
@@ -17501,7 +17501,7 @@
       </c>
       <c r="Q190" t="inlineStr">
         <is>
-          <t>wojcik.joanna@icloud.com</t>
+          <t>wojcik.joanna@onet.pl</t>
         </is>
       </c>
       <c r="R190" t="inlineStr">
@@ -17593,7 +17593,7 @@
       </c>
       <c r="Q191" t="inlineStr">
         <is>
-          <t>pawelkowalczyk@gmail.com</t>
+          <t>pawelkowalczyk@interia.pl</t>
         </is>
       </c>
       <c r="R191" t="inlineStr">
@@ -17685,7 +17685,7 @@
       </c>
       <c r="Q192" t="inlineStr">
         <is>
-          <t>magdalena_kaminska@wp.pl</t>
+          <t>magdalena_kaminska@o2.pl</t>
         </is>
       </c>
       <c r="R192" t="inlineStr">
@@ -17777,7 +17777,7 @@
       </c>
       <c r="Q193" t="inlineStr">
         <is>
-          <t>robert.lewandowski78@onet.pl</t>
+          <t>robert.lewandowski78@proton.me</t>
         </is>
       </c>
       <c r="R193" t="inlineStr">
@@ -17869,7 +17869,7 @@
       </c>
       <c r="Q194" t="inlineStr">
         <is>
-          <t>agnieszka.zielinska@wp</t>
+          <t>agnieszka.zielinska@outlook.com</t>
         </is>
       </c>
       <c r="R194" t="inlineStr">
@@ -17961,7 +17961,7 @@
       </c>
       <c r="Q195" t="inlineStr">
         <is>
-          <t>w.szymanski@o2.pl</t>
+          <t>w.szymanski@yahoo.com</t>
         </is>
       </c>
       <c r="R195" t="inlineStr">
@@ -18053,7 +18053,7 @@
       </c>
       <c r="Q196" t="inlineStr">
         <is>
-          <t>dabrowska.justyna@proton.me</t>
+          <t>dabrowska.justyna@icloud.com</t>
         </is>
       </c>
       <c r="R196" t="inlineStr">
@@ -18145,7 +18145,7 @@
       </c>
       <c r="Q197" t="inlineStr">
         <is>
-          <t>piotrmazur@outlook.com</t>
+          <t>piotrmazur@gmail.com</t>
         </is>
       </c>
       <c r="R197" t="inlineStr">
@@ -18237,7 +18237,7 @@
       </c>
       <c r="Q198" t="inlineStr">
         <is>
-          <t>maria_krawczyk@yahoo.com</t>
+          <t>maria_krawczyk@wp.pl</t>
         </is>
       </c>
       <c r="R198" t="inlineStr">
@@ -18329,7 +18329,7 @@
       </c>
       <c r="Q199" t="inlineStr">
         <is>
-          <t>@michal.wozniak84.invalid</t>
+          <t>email.20740197@onet.pl</t>
         </is>
       </c>
       <c r="R199" t="inlineStr">
@@ -18421,7 +18421,7 @@
       </c>
       <c r="Q200" t="inlineStr">
         <is>
-          <t>joanna.jankowska@gmail.com</t>
+          <t>joanna.jankowska@interia.pl</t>
         </is>
       </c>
       <c r="R200" t="inlineStr">
@@ -18513,7 +18513,7 @@
       </c>
       <c r="Q201" t="inlineStr">
         <is>
-          <t>p.grabowski@wp.pl</t>
+          <t>p.grabowski@o2.pl</t>
         </is>
       </c>
       <c r="R201" t="inlineStr">

</xml_diff>